<commit_message>
Add FOT payroll positions from historical FEM sheets
Extract job titles from dedicated FOT worksheets across 20 historical FEM
files and add 54 positions under 'Затраты по заработной плате' (OPEX).

Co-authored-by: TemeshevProject <TemeshevProject@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/fem-artifacts/main_artifacts_updated.xlsx
+++ b/fem-artifacts/main_artifacts_updated.xlsx
@@ -23927,7 +23927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z148"/>
+  <dimension ref="A1:Z202"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.42578125" defaultRowHeight="15"/>
   <cols>
     <col width="7.7109375" customWidth="1" style="74" min="1" max="1"/>
@@ -27829,12 +27829,12 @@
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Билеты (ж.д. сообщение, плацкарт, 2 направления)</t>
+          <t>Менеджер проектов</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -27844,22 +27844,22 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M88" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Билеты (ж.д. сообщение, купе, 2 направления)</t>
+          <t>Технический директор</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -27869,22 +27869,22 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M89" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Билеты (авиа сообщение,  2 направления)</t>
+          <t>Инженер контроля качества</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -27894,22 +27894,22 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M90" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Проживание (сутки гостиница для производств.сотрудников)</t>
+          <t>Бухгалтер</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -27919,22 +27919,22 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M91" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Проживание (сутки гостиница для АУП)</t>
+          <t>Директор филиала</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -27944,22 +27944,22 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M92" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Суточные (6 мрп)</t>
+          <t>Юрист</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M93" t="n">
@@ -27979,12 +27979,12 @@
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>7. Расчет экспл.расх</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ДТ для ДГУ</t>
+          <t>Инспектор по кадрам</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -27994,11 +27994,11 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M94" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="95">
@@ -28009,7 +28009,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Охрана</t>
+          <t>Билеты (ж.д. сообщение, плацкарт, 2 направления)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -28023,7 +28023,7 @@
         </is>
       </c>
       <c r="M95" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96">
@@ -28034,7 +28034,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Канц. Товары</t>
+          <t>Билеты (ж.д. сообщение, купе, 2 направления)</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -28048,7 +28048,7 @@
         </is>
       </c>
       <c r="M96" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="97">
@@ -28059,7 +28059,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Хоз. Товары</t>
+          <t>Билеты (авиа сообщение,  2 направления)</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -28073,7 +28073,7 @@
         </is>
       </c>
       <c r="M97" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="98">
@@ -28084,7 +28084,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Клининговые услуги</t>
+          <t>Проживание (сутки гостиница для производств.сотрудников)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -28098,7 +28098,7 @@
         </is>
       </c>
       <c r="M98" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="99">
@@ -28109,7 +28109,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>ГСМ для сотрудников</t>
+          <t>Проживание (сутки гостиница для АУП)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -28119,197 +28119,197 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Туркестан фин 04.11.2025.xlsx::5. Экспл; ФЭМ №1 (Павлодар).xlsx::5. Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M99" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>Оснащение рабочих мест Ситуационного центра</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Оснащение оборудованием ситуационного центра</t>
+          <t>Суточные (6 мрп)</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>4. Шу_ФЭМ.xlsx::3. Инвест; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ №1 (Павлодар).xlsx::3. Инвест; ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M100" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>Инвест</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Метеостанция: PM 2.5, PM10, ветер, температура, осадки</t>
+          <t>Водитель логист</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ; ФЭМ_проекта_Жетысу_final.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M101" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>Инвест</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Планшет, принтер, ПО</t>
+          <t>Офис-менеджер</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ; ФЭМ_проекта_Жетысу_final.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M102" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
+          <t>7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Затраты на оборудование для интеграции на 1 существующую камеру</t>
+          <t>ДТ для ДГУ</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M103" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>АПК "Сергек.Линейный"</t>
+          <t>Охрана</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M104" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>АПК "Сергек.Перекресток"</t>
+          <t>Канц. Товары</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M105" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>монтаж оборудования для интеграции</t>
+          <t>Хоз. Товары</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M106" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>7. Расчет экспл.расх</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Канал передачи данных - центральный узел</t>
+          <t>Экономист</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -28319,97 +28319,97 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх; ФЭМ №1 (Павлодар).xlsx::5. Экспл; ФЭМ_Туркестан_1006.xlsx::Экспл</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M107" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>Оснащение рабочих мест Ситуационного центра</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Мобильное рабочее место + лицензия MDM</t>
+          <t>Менеджер отдела закупа</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>4. Шу_ФЭМ.xlsx::3. Инвест; ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M108" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>Центр обработки и анализа данных</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Система серверов процессинга и аналитики, включая ПО</t>
+          <t>Клининговые услуги</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M109" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>Центр обработки и анализа данных</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Система серверов хранения данных, включая ПО</t>
+          <t>ГСМ для сотрудников</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
+          <t>4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Туркестан фин 04.11.2025.xlsx::5. Экспл; ФЭМ №1 (Павлодар).xlsx::5. Экспл</t>
         </is>
       </c>
       <c r="M110" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
+          <t>Оснащение рабочих мест Ситуационного центра</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>монтаж оборудования линейных участков</t>
+          <t>Оснащение оборудованием ситуационного центра</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -28419,47 +28419,47 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
+          <t>4. Шу_ФЭМ.xlsx::3. Инвест; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ №1 (Павлодар).xlsx::3. Инвест; ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M111" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>монтаж оборудования перекрестков</t>
+          <t>Старший инженер контроля качества</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ_проекта_Жетысу_final.xlsx::6. ФОТ; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M112" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>4.CAPEX</t>
+          <t>Инвест</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Инструменты и средства индивидуальной защиты</t>
+          <t>Метеостанция: PM 2.5, PM10, ветер, температура, осадки</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -28469,22 +28469,22 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ №1 (Павлодар).xlsx::3. Инвест; ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
         </is>
       </c>
       <c r="M113" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Инвест</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплекс на линейном участке</t>
+          <t>Планшет, принтер, ПО</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -28494,22 +28494,22 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
         </is>
       </c>
       <c r="M114" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплекс на перекрестке</t>
+          <t>Затраты на оборудование для интеграции на 1 существующую камеру</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -28519,11 +28519,11 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
         </is>
       </c>
       <c r="M115" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="116">
@@ -28534,7 +28534,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Мобильное рабочее место</t>
+          <t>АПК "Сергек.Линейный"</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -28544,22 +28544,22 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M116" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>Инструменты и средства индивидуальной защиты</t>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Мобильный интеллектуальный АПК</t>
+          <t>АПК "Сергек.Перекресток"</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -28569,22 +28569,22 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M117" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>Инструменты и средства индивидуальной защиты</t>
+          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Транспортный двойник города</t>
+          <t>монтаж оборудования для интеграции</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -28594,22 +28594,22 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест; ФЭМ_Атырау.xlsx::Инвест</t>
         </is>
       </c>
       <c r="M118" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>Экспл</t>
+          <t>7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Аренда ЦОД</t>
+          <t>Канал передачи данных - центральный узел</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -28619,36 +28619,36 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх; ФЭМ №1 (Павлодар).xlsx::5. Экспл; ФЭМ_Туркестан_1006.xlsx::Экспл</t>
         </is>
       </c>
       <c r="M119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>Экспл</t>
+          <t>Оснащение рабочих мест Ситуационного центра</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Коммунальные расходы (электроэнергия)</t>
+          <t>Мобильное рабочее место + лицензия MDM</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
+          <t>4. Шу_ФЭМ.xlsx::3. Инвест; ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M120" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Сервера хранения данных, 1 ПТб</t>
+          <t>Система серверов процессинга и аналитики, включая ПО</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -28669,22 +28669,22 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>ФЭМ_Атырау.xlsx::Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
         </is>
       </c>
       <c r="M121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>Инвест</t>
+          <t>Центр обработки и анализа данных</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Расходные материалы на подключение к сети</t>
+          <t>Система серверов хранения данных, включая ПО</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -28694,22 +28694,22 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>ФЭМ_Атырау.xlsx::Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
         </is>
       </c>
       <c r="M122" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплек "Сергек. Патруль BOX"</t>
+          <t>монтаж оборудования линейных участков</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -28719,11 +28719,11 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
         </is>
       </c>
       <c r="M123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="124">
@@ -28734,7 +28734,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Монтаж АПК патруль</t>
+          <t>монтаж оборудования перекрестков</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -28744,22 +28744,22 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
+          <t>ФЭМ ИСХОДНАЯ.xlsx::Инвест; ФЭМ ИТОГ до ноября24.xlsx::Инвест; ФЭМ_16_07_приложение_к_доп_согл.xlsx::Инвест; ФЭМ_Астана (4).xlsx::Инвест</t>
         </is>
       </c>
       <c r="M124" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>5. Экспл</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Обслуживание  АПК "Патруль"</t>
+          <t>Ведущий инженер контроля качества</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -28769,36 +28769,36 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>ФЭМ_проекта_Жетысу_final.xlsx::5. Экспл; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::5. Экспл; ФЭМ_проекта_Курмангазы v.8.xlsx::5. Экспл</t>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
         </is>
       </c>
       <c r="M125" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Счетчики АСКУЭ для АПК "Сергек"</t>
+          <t>Инженер сетей</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ; финал_ФЭМ_проекта_Туркестан_расширение_и_продление_v_2_с_помесячн_графиком.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M126" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127">
@@ -28809,7 +28809,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Универсальный шлюз безопасности (NGFW)</t>
+          <t>Инструменты и средства индивидуальной защиты</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -28819,22 +28819,22 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ №1 (Павлодар).xlsx::3. Инвест; ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Монтаж АПК "Сергек.Линейный"</t>
+          <t>Аппаратно-программный комплекс на линейном участке</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -28844,22 +28844,22 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Монтаж АПК "Сергек.Перекресток"</t>
+          <t>Аппаратно-программный комплекс на перекрестке</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -28869,11 +28869,11 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M129" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="130">
@@ -28884,7 +28884,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Подключение каналов связи (АПК "Сергек")</t>
+          <t>Мобильное рабочее место</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -28894,22 +28894,22 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Инструменты и средства индивидуальной защиты</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Поверка (АПК "Сергек")</t>
+          <t>Мобильный интеллектуальный АПК</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -28919,22 +28919,22 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t>Для CAPEX</t>
+          <t>Инструменты и средства индивидуальной защиты</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Зарядное устройство С 4/36-90 230V box</t>
+          <t>Транспортный двойник города</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -28944,22 +28944,22 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::Для CAPEX; ФЭМ Костанай.xlsx::Для CAPEX</t>
+          <t>Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::3. Инвест; ФЭМ ДС №2 Алмобл 26.02 .xlsx::3. Инвест; ФЭМ_ДС_09_06_2025_для_нового_состава_2 (2).xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Экспл</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Канал передачи данных - АПК "Сергек.Линейный"</t>
+          <t>Аренда ЦОД</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -28969,22 +28969,22 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
         </is>
       </c>
       <c r="M133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="134">
       <c r="B134" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Экспл</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Канал передачи данных - АПК "Сергек.Перекресток"</t>
+          <t>Коммунальные расходы (электроэнергия)</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -28994,47 +28994,47 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
         </is>
       </c>
       <c r="M134" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t>Центр обработки и анализа данных</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Резервный сервер</t>
+          <t>Ведущий менеджер проектов</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>4. Шу_ФЭМ.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест</t>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
         </is>
       </c>
       <c r="M135" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="136">
       <c r="B136" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Центр обработки и анализа данных</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Мобильное рабочее место "Сергек"</t>
+          <t>Сервера хранения данных, 1 ПТб</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -29044,47 +29044,47 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>ФЭМ №1 (Павлодар).xlsx::3. Инвест; ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
+          <t>ФЭМ_Атырау.xlsx::Инвест</t>
         </is>
       </c>
       <c r="M136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Инвест</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Распределение расходов административно-управленческого персонала,осуществляющего поддержку проекта Астана - Сергек ( прочие расходы)</t>
+          <t>Расходные материалы на подключение к сети</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>ФЭМ_Астана (4).xlsx::Обсл; ФЭМ_Астана (4).xlsx::Экспл</t>
+          <t>ФЭМ_Атырау.xlsx::Инвест</t>
         </is>
       </c>
       <c r="M137" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>Инвест</t>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Видеостена под ключ</t>
+          <t>Аппаратно-программный комплек "Сергек. Патруль BOX"</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -29094,22 +29094,22 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>ФЭМ_Атырау.xlsx::Инвест</t>
+          <t>ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M138" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплекс "Сергек. Трасса" v4.0</t>
+          <t>Монтаж АПК патруль</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -29119,36 +29119,36 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
+          <t>ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
         </is>
       </c>
       <c r="M139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="140">
       <c r="B140" t="inlineStr">
         <is>
-          <t>4.CAPEX</t>
+          <t>5. Экспл</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Видеостена (13500х6500), под ключ</t>
+          <t>Обслуживание  АПК "Патруль"</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX</t>
+          <t>ФЭМ_проекта_Жетысу_final.xlsx::5. Экспл; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::5. Экспл; ФЭМ_проекта_Курмангазы v.8.xlsx::5. Экспл</t>
         </is>
       </c>
       <c r="M140" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="141">
@@ -29159,7 +29159,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплекс "Сергек. Патруль"</t>
+          <t>Счетчики АСКУЭ для АПК "Сергек"</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -29169,22 +29169,22 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>4. Шу_ФЭМ.xlsx::3. Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
         </is>
       </c>
       <c r="M141" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>4.CAPEX</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплекс "Сергек. Трасса"</t>
+          <t>Универсальный шлюз безопасности (NGFW)</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -29194,47 +29194,47 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>4. Шу_ФЭМ.xlsx::3. Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
         </is>
       </c>
       <c r="M142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="143">
       <c r="B143" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Распределение расходов административно-управленческого персонала,осуществляющего поддержку проекта Астана - Сергек за  декабрь 2022г. ( прочие расходы)</t>
+          <t>Монтаж АПК "Сергек.Линейный"</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>ФЭМ ИТОГ до ноября24.xlsx::Обсл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
         </is>
       </c>
       <c r="M143" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="144">
       <c r="B144" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Стоимость монтажных работ и услуг для запуска проекта</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>АПК "Сергек" на линейных участках</t>
+          <t>Монтаж АПК "Сергек.Перекресток"</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -29244,11 +29244,11 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
         </is>
       </c>
       <c r="M144" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
@@ -29259,7 +29259,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>АПК "Сергек" на перекрестках</t>
+          <t>Подключение каналов связи (АПК "Сергек")</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -29269,11 +29269,11 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>ФЭМ Костанай.xlsx::4.CAPEX</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
         </is>
       </c>
       <c r="M145" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="146">
@@ -29284,7 +29284,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплекс "Сергек. Трассы"</t>
+          <t>Поверка (АПК "Сергек")</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -29294,22 +29294,22 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX; ФЭМ Костанай.xlsx::4.CAPEX</t>
         </is>
       </c>
       <c r="M146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Для CAPEX</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Аппаратно-программный комплекс "Сергек. Линейный участок" v4.0 на трассах</t>
+          <t>Зарядное устройство С 4/36-90 230V box</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -29319,35 +29319,1385 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::Для CAPEX; ФЭМ Костанай.xlsx::Для CAPEX</t>
         </is>
       </c>
       <c r="M147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148">
       <c r="B148" t="inlineStr">
         <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Старший специалист по тех. поддержке</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M148" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Специалист по тех. поддержке</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M149" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Менеджер по технике безопасности</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M150" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Калибровщик</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M151" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Логист тестировщик</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M152" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" t="inlineStr">
+        <is>
           <t>Аппаратно-программные комплексы "Сергек"</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Канал передачи данных - АПК "Сергек.Линейный"</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+        </is>
+      </c>
+      <c r="M153" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Канал передачи данных - АПК "Сергек.Перекресток"</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+        </is>
+      </c>
+      <c r="M154" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Центр обработки и анализа данных</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Резервный сервер</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>4. Шу_ФЭМ.xlsx::3. Инвест; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест</t>
+        </is>
+      </c>
+      <c r="M155" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Заместитель директора филиала</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M156" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Менеджер мониторинга</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M157" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Ассистент руководителя</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M158" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Главный инженер контроля качества</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M159" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Ведущий инженер по сервисам</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M160" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Инженер по сервисам</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M161" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Логист</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M162" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Генеральный директор</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M163" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Исполнительный директор по финансам и обеспечению</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M164" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Советник по информационной безопасности</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M165" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Директор по финансовым  вопросам</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M166" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Главный финансовый менеджер</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M167" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Финансовый менеджер</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M168" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Главный бухгалтер</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M169" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Директор по правовым вопросам</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M170" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Заместитель директора по правовым вопросам</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M171" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Главный юрист</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M172" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Старший юрист</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M173" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Менеджер по безопасности</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M174" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Главный менеджер по ИБ</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M175" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Корпоративный секретарь</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Ассистент</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M177" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Заведующий складом</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M178" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Директор по управлению проектами</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M179" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Заместитель директора Департамента</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M180" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Аналитик по эффективности и рискам</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M181" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Младший менеджер проектов</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M182" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Начальник отдела по связям с общественностью и СМИ</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M183" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Мобильное рабочее место "Сергек"</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>ФЭМ №1 (Павлодар).xlsx::3. Инвест; ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
+        </is>
+      </c>
+      <c r="M184" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Распределение расходов административно-управленческого персонала,осуществляющего поддержку проекта Астана - Сергек ( прочие расходы)</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>ФЭМ_Астана (4).xlsx::Обсл; ФЭМ_Астана (4).xlsx::Экспл</t>
+        </is>
+      </c>
+      <c r="M185" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Инвест</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Видеостена под ключ</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>ФЭМ_Атырау.xlsx::Инвест</t>
+        </is>
+      </c>
+      <c r="M186" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Аппаратно-программный комплекс "Сергек. Трасса" v4.0</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::3. Инвест; ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
+        </is>
+      </c>
+      <c r="M187" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Главный инженер</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M188" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Старший бригадир</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M189" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Инженер ОКК</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M190" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Бригадир</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M191" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Старший монтажник</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M192" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Младший монтажник</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M193" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>4.CAPEX</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Видеостена (13500х6500), под ключ</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::4.CAPEX</t>
+        </is>
+      </c>
+      <c r="M194" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Аппаратно-программный комплекс "Сергек. Патруль"</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>4. Шу_ФЭМ.xlsx::3. Инвест</t>
+        </is>
+      </c>
+      <c r="M195" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Аппаратно-программный комплекс "Сергек. Трасса"</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>4. Шу_ФЭМ.xlsx::3. Инвест</t>
+        </is>
+      </c>
+      <c r="M196" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Распределение расходов административно-управленческого персонала,осуществляющего поддержку проекта Астана - Сергек за  декабрь 2022г. ( прочие расходы)</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::Обсл</t>
+        </is>
+      </c>
+      <c r="M197" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>АПК "Сергек" на линейных участках</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>ФЭМ Костанай.xlsx::4.CAPEX</t>
+        </is>
+      </c>
+      <c r="M198" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>АПК "Сергек" на перекрестках</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>ФЭМ Костанай.xlsx::4.CAPEX</t>
+        </is>
+      </c>
+      <c r="M199" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Аппаратно-программный комплекс "Сергек. Трассы"</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>ФЭМ №2 (Павлодар).xlsx::3. Инвест</t>
+        </is>
+      </c>
+      <c r="M200" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Аппаратно-программный комплекс "Сергек. Линейный участок" v4.0 на трассах</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Жетысу_final.xlsx::3. Инвест</t>
+        </is>
+      </c>
+      <c r="M201" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
         <is>
           <t>Аппаратно-программный комплекс "Сергек. Lite"</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr">
+      <c r="D202" t="inlineStr">
         <is>
           <t>CAPEX</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr">
+      <c r="L202" t="inlineStr">
         <is>
           <t>ФЭМ_проекта_Курмангазы v.8.xlsx::3. Инвест</t>
         </is>
       </c>
-      <c r="M148" t="n">
+      <c r="M202" t="n">
         <v>1</v>
       </c>
     </row>
@@ -34645,7 +35995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M67"/>
+  <dimension ref="B2:M121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -36684,12 +38034,12 @@
     <row r="48">
       <c r="B48" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Билеты (ж.д. сообщение, плацкарт, 2 направления)</t>
+          <t>Менеджер проектов</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -36699,22 +38049,22 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M48" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Билеты (ж.д. сообщение, купе, 2 направления)</t>
+          <t>Технический директор</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -36724,22 +38074,22 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M49" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Билеты (авиа сообщение,  2 направления)</t>
+          <t>Инженер контроля качества</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -36749,22 +38099,22 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M50" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Проживание (сутки гостиница для производств.сотрудников)</t>
+          <t>Бухгалтер</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -36774,22 +38124,22 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M51" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Проживание (сутки гостиница для АУП)</t>
+          <t>Директор филиала</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -36799,22 +38149,22 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M52" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>Экономические предположения</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Суточные (6 мрп)</t>
+          <t>Юрист</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -36824,7 +38174,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
         </is>
       </c>
       <c r="M53" t="n">
@@ -36834,12 +38184,12 @@
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>7. Расчет экспл.расх</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ДТ для ДГУ</t>
+          <t>Инспектор по кадрам</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -36849,11 +38199,11 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M54" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55">
@@ -36864,7 +38214,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Охрана</t>
+          <t>Билеты (ж.д. сообщение, плацкарт, 2 направления)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -36878,7 +38228,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56">
@@ -36889,7 +38239,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Канц. Товары</t>
+          <t>Билеты (ж.д. сообщение, купе, 2 направления)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -36903,7 +38253,7 @@
         </is>
       </c>
       <c r="M56" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57">
@@ -36914,7 +38264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Хоз. Товары</t>
+          <t>Билеты (авиа сообщение,  2 направления)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -36928,7 +38278,7 @@
         </is>
       </c>
       <c r="M57" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58">
@@ -36939,7 +38289,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Клининговые услуги</t>
+          <t>Проживание (сутки гостиница для производств.сотрудников)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -36953,7 +38303,7 @@
         </is>
       </c>
       <c r="M58" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="59">
@@ -36964,7 +38314,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ГСМ для сотрудников</t>
+          <t>Проживание (сутки гостиница для АУП)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -36974,22 +38324,22 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Туркестан фин 04.11.2025.xlsx::5. Экспл; ФЭМ №1 (Павлодар).xlsx::5. Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M59" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>7. Расчет экспл.расх</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Канал передачи данных - центральный узел</t>
+          <t>Суточные (6 мрп)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -36999,22 +38349,22 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх; ФЭМ №1 (Павлодар).xlsx::5. Экспл; ФЭМ_Туркестан_1006.xlsx::Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M60" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t>Экспл</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Аренда ЦОД</t>
+          <t>Водитель логист</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -37024,22 +38374,22 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ; ФЭМ_проекта_Жетысу_final.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M61" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>Экспл</t>
+          <t>Затраты по заработной плате</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Коммунальные расходы (электроэнергия)</t>
+          <t>Офис-менеджер</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -37049,22 +38399,22 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ; ФЭМ_проекта_Жетысу_final.xlsx::6. ФОТ</t>
         </is>
       </c>
       <c r="M62" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>5. Экспл</t>
+          <t>7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Обслуживание  АПК "Патруль"</t>
+          <t>ДТ для ДГУ</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -37074,22 +38424,22 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>ФЭМ_проекта_Жетысу_final.xlsx::5. Экспл; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::5. Экспл; ФЭМ_проекта_Курмангазы v.8.xlsx::5. Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M63" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Канал передачи данных - АПК "Сергек.Линейный"</t>
+          <t>Охрана</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -37099,22 +38449,22 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M64" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Канал передачи данных - АПК "Сергек.Перекресток"</t>
+          <t>Канц. Товары</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -37124,22 +38474,22 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M65" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
-          <t>Аппаратно-программные комплексы "Сергек"</t>
+          <t>Экономические предположения</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Распределение расходов административно-управленческого персонала,осуществляющего поддержку проекта Астана - Сергек ( прочие расходы)</t>
+          <t>Хоз. Товары</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -37149,35 +38499,1385 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>ФЭМ_Астана (4).xlsx::Обсл; ФЭМ_Астана (4).xlsx::Экспл</t>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
         </is>
       </c>
       <c r="M66" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Экономист</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Менеджер отдела закупа</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-04-21 Прил 3 ФЭМ_Акмола (35 млрд).xlsx::4.1.ФОТ; 2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Экономические предположения</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Клининговые услуги</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; 4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Экономические предположения</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>ГСМ для сотрудников</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>4. Шу_ФЭМ.xlsx::5. Экспл; Прил_ФЭМ_Алм_обл_расширение_тарифы_для_3_ПК_19_03_2025_1.xlsx::5. Экспл; ФЭМ ДС №2 Алмобл 26.02 .xlsx::5. Экспл; ФЭМ Туркестан фин 04.11.2025.xlsx::5. Экспл; ФЭМ №1 (Павлодар).xlsx::5. Экспл</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Старший инженер контроля качества</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; 4. Шу_ФЭМ.xlsx::6. ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ; ФЭМ_проекта_Жетысу_final.xlsx::6. ФОТ; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>7. Расчет экспл.расх</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Канал передачи данных - центральный узел</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх; ФЭМ №1 (Павлодар).xlsx::5. Экспл; ФЭМ_Туркестан_1006.xlsx::Экспл</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Ведущий инженер контроля качества</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Инженер сетей</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>ФЭМ Туркестан фин 04.11.2025.xlsx::6. ФОТ; финал_ФЭМ_проекта_Туркестан_расширение_и_продление_v_2_с_помесячн_графиком.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M74" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Экспл</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Аренда ЦОД</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
+        </is>
+      </c>
+      <c r="M75" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Экспл</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Коммунальные расходы (электроэнергия)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::Экспл; ФЭМ_Астана (4).xlsx::Экспл</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Ведущий менеджер проектов</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M77" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>5. Экспл</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Обслуживание  АПК "Патруль"</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Жетысу_final.xlsx::5. Экспл; ФЭМ_проекта_Кульсары_Расширение_новый_состав_1_8.xlsx::5. Экспл; ФЭМ_проекта_Курмангазы v.8.xlsx::5. Экспл</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Старший специалист по тех. поддержке</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Специалист по тех. поддержке</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M80" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Менеджер по технике безопасности</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Калибровщик</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Логист тестировщик</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::5.Расчет ФОТ; ФЭМ Костанай.xlsx::5.Расчет ФОТ</t>
+        </is>
+      </c>
+      <c r="M83" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="inlineStr">
+        <is>
           <t>Аппаратно-программные комплексы "Сергек"</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Канал передачи данных - АПК "Сергек.Линейный"</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+        </is>
+      </c>
+      <c r="M84" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Канал передачи данных - АПК "Сергек.Перекресток"</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2_ФЭМ_Костанай_3,5млрд_v3_в_коротком_виде2.xlsx::7. Расчет экспл.расх; ФЭМ Костанай.xlsx::7. Расчет экспл.расх</t>
+        </is>
+      </c>
+      <c r="M85" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Заместитель директора филиала</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M86" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Менеджер мониторинга</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M87" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Ассистент руководителя</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M88" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Главный инженер контроля качества</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M89" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Ведущий инженер по сервисам</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Инженер по сервисам</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M91" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Логист</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M92" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Генеральный директор</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M93" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Исполнительный директор по финансам и обеспечению</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M94" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Советник по информационной безопасности</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M95" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Директор по финансовым  вопросам</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M96" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Главный финансовый менеджер</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M97" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Финансовый менеджер</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M98" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Главный бухгалтер</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M99" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Директор по правовым вопросам</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M100" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Заместитель директора по правовым вопросам</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M101" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Главный юрист</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M102" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Старший юрист</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M103" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Менеджер по безопасности</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M104" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Главный менеджер по ИБ</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M105" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Корпоративный секретарь</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M106" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Ассистент</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M107" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Заведующий складом</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M108" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Директор по управлению проектами</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M109" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Заместитель директора Департамента</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M110" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Аналитик по эффективности и рискам</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M111" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Младший менеджер проектов</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M112" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Начальник отдела по связям с общественностью и СМИ</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>ФЭМ ИТОГ до ноября24.xlsx::ФОТ н; ФЭМ_Астана (4).xlsx::ФОТ н</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Распределение расходов административно-управленческого персонала,осуществляющего поддержку проекта Астана - Сергек ( прочие расходы)</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>ФЭМ_Астана (4).xlsx::Обсл; ФЭМ_Астана (4).xlsx::Экспл</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Главный инженер</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M115" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Старший бригадир</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M116" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Инженер ОКК</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Бригадир</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M118" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Старший монтажник</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M119" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Затраты по заработной плате</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Младший монтажник</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>ФЭМ_проекта_Курмангазы v.8.xlsx::6. ФОТ</t>
+        </is>
+      </c>
+      <c r="M120" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Аппаратно-программные комплексы "Сергек"</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
         <is>
           <t>Распределение расходов административно-управленческого персонала,осуществляющего поддержку проекта Астана - Сергек за  декабрь 2022г. ( прочие расходы)</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D121" t="inlineStr">
         <is>
           <t>OPEX</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr">
+      <c r="L121" t="inlineStr">
         <is>
           <t>ФЭМ ИТОГ до ноября24.xlsx::Обсл</t>
         </is>
       </c>
-      <c r="M67" t="n">
+      <c r="M121" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>